<commit_message>
Fix Wind audit strip IRR/MOIC references
Model_6_Wind.xlsx + Drill_6_Wind.xlsx:
- R8 (Levered IRR): =D128 → =D131 (points to actual IRR formula)
- R9 (MOIC): =D129 → =D132 (points to actual MOIC formula)

ZIP SHA256: 09aeff31b30cd0cca2728b04afc85daa11cd7132b63e1cab42a5f9bd92ade1e5

Full verification complete:
✓ 6 Models: All have IRR formulas, QA checks, no errors
✓ 6 Drills: All have DRILL MODE note, no errors
✓ Supporting files: Present and accessible
</commit_message>
<xml_diff>
--- a/deliverables/deliverables-20260120-0030/Drill_6_Wind.xlsx
+++ b/deliverables/deliverables-20260120-0030/Drill_6_Wind.xlsx
@@ -2197,7 +2197,7 @@
         </is>
       </c>
       <c r="D8" s="7">
-        <f>D128</f>
+        <f>D131</f>
         <v/>
       </c>
     </row>
@@ -2213,7 +2213,7 @@
         </is>
       </c>
       <c r="D9" s="7">
-        <f>D129</f>
+        <f>D132</f>
         <v/>
       </c>
     </row>

</xml_diff>